<commit_message>
Fase 3 oppstart: litteratur, data, intervjuguide og benchmarkanalyse
- 33 PDF-referanser lagt til i 003 references/ (34 kilder totalt)
- Litteraturliste oppdatert og verifisert
- Intervjuguide opprettet (utkast) og møtereferat Midt-Norge 110 (15. mars)
- Benchmarkskript og figurer (MOB 2018-2025) lagt til
- status.md v1.1: datagrunnlag, BRIS-begrensning og intervjulogg oppdatert
- Gantt og rapport oppdatert
- Kursmateriale fase 2 og 3 samt KI-erklæringsmal lagt til

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
+++ b/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\runeg\OneDrive\Documents\Skole utdanning\Logistikk studie\LOG650 LOGISTIKK OG KI\G20-rune-individuell\012 fase 2 - plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be25ac4905db4876/Documents/Skole utdanning/Logistikk studie/LOG650 LOGISTIKK OG KI/G20-rune-individuell/012 fase 2 - plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD33CF9-27BD-4424-8BC7-EFD69435E682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="13_ncr:1_{CCD33CF9-27BD-4424-8BC7-EFD69435E682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCFC1ABC-F1D7-464C-8866-5E795743F36F}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,11 +17,12 @@
     <sheet name="Veiledning" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="319">
   <si>
     <t>Nr</t>
   </si>
@@ -984,7 +985,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1015,8 +1016,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1026,11 +1032,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD6E4F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -1045,11 +1046,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAD3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFEA9999"/>
       </patternFill>
     </fill>
@@ -1060,16 +1056,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE5CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1107,64 +1099,424 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperkobling" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="19">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF999999"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF999999"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F3864"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF999999"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF999999"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1175,6 +1527,30 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A02DC60A-3F25-4919-ADF0-970C442FCB0A}" name="Tabell1" displayName="Tabell1" ref="A1:O39" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15">
+  <autoFilter ref="A1:O39" xr:uid="{A02DC60A-3F25-4919-ADF0-970C442FCB0A}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{B05B6C21-03AB-4D4C-8F3F-2AD82AF26B8B}" name="Nr" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{A24D361C-4CF0-40EC-93A1-180C5AACA04C}" name="Kategori" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B99C806F-A0B6-4046-A219-B84628DB1B24}" name="Forfatter(e)" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{20BC4260-9346-4BE8-948B-A4A787262396}" name="Tittel" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{4840409B-A22A-408B-9506-AEB0CD4384DA}" name="År" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{FC073743-1A85-4E32-9515-7D29CD222999}" name="Publikasjonskanal" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{D6767AA9-6F03-4BCA-BC8D-6B11026CCD67}" name="Type" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{C49687EB-EC67-423B-8DF2-6DD8A5F02813}" name="Relevans for prosjektet" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{A41AD885-99DF-443B-BD38-B2A568569A21}" name="Verifisert?" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{26525674-05E5-4B7D-8857-C25465E6FA91}" name="URL / DOI" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{9C4AA926-BBEA-43D8-AD0A-2DDCDE5E8DB0}" name="Tilgjengelighet" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{67D71043-E968-4FF3-86B0-2E22B48FF094}" name="Lastet ned" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{BD0D5372-1048-45A4-85B3-7BE5372859DB}" name="Brukt i rapport?" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{885DA868-5D93-4E2A-B726-139ACD494513}" name="APA 7th referanse" dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{C8728198-2E5E-4777-8C70-86B9E52AAF54}" name="Notater" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1476,1206 +1852,1196 @@
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="35" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="8" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="12" max="12" width="11.53125" customWidth="1"/>
+    <col min="13" max="13" width="16.19921875" customWidth="1"/>
     <col min="14" max="14" width="55" customWidth="1"/>
     <col min="15" max="15" width="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-    </row>
-    <row r="3" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="2">
+    </row>
+    <row r="3" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="8">
         <v>2003</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2" t="s">
+      <c r="M3" s="8"/>
+      <c r="N3" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="2"/>
-    </row>
-    <row r="4" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="2">
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="8">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="8">
         <v>2005</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2" t="s">
+      <c r="L4" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="2"/>
-    </row>
-    <row r="5" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="2">
+      <c r="O4" s="8"/>
+    </row>
+    <row r="5" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="8">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="8">
         <v>1981</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2" t="s">
+      <c r="L5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="2">
+      <c r="O5" s="8"/>
+    </row>
+    <row r="6" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="8">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="8">
         <v>2002</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2" t="s">
+      <c r="L6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="O6" s="2"/>
-    </row>
-    <row r="7" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="2">
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="8">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="8">
         <v>2007</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2" t="s">
+      <c r="L7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="2">
+      <c r="O7" s="8"/>
+    </row>
+    <row r="8" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="8">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="8">
         <v>2008</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2" t="s">
+      <c r="L8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="2">
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="8">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="8">
         <v>2016</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2" t="s">
+      <c r="L9" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="2">
+      <c r="O9" s="8"/>
+    </row>
+    <row r="10" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="8">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="8">
         <v>2008</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2" t="s">
+      <c r="L10" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="2">
+      <c r="O10" s="8"/>
+    </row>
+    <row r="11" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="8">
         <v>9</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="8">
         <v>2011</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="J11" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2" t="s">
+      <c r="L11" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="O11" s="2"/>
+      <c r="O11" s="8"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-    </row>
-    <row r="13" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="5">
+    </row>
+    <row r="13" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="8">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="8">
         <v>2018</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5" t="s">
+      <c r="L13" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="O13" s="5"/>
-    </row>
-    <row r="14" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="5">
+      <c r="O13" s="8"/>
+    </row>
+    <row r="14" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="8">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="8">
         <v>2017</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5" t="s">
+      <c r="L14" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="O14" s="5"/>
-    </row>
-    <row r="15" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="5">
+      <c r="O14" s="8"/>
+    </row>
+    <row r="15" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="8">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="8">
         <v>2018</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="K15" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5" t="s">
+      <c r="L15" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="O15" s="5"/>
-    </row>
-    <row r="16" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="5">
+      <c r="O15" s="8"/>
+    </row>
+    <row r="16" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="8">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="8">
         <v>2013</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="J16" s="5" t="s">
+      <c r="J16" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="K16" s="5" t="s">
+      <c r="K16" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5" t="s">
+      <c r="L16" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="O16" s="5"/>
-    </row>
-    <row r="17" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="5">
+      <c r="O16" s="8"/>
+    </row>
+    <row r="17" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="8">
         <v>14</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="8">
         <v>2002</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J17" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="K17" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5" t="s">
+      <c r="L17" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="O17" s="5"/>
-    </row>
-    <row r="18" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="5">
+      <c r="O17" s="8"/>
+    </row>
+    <row r="18" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="8">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="8">
         <v>2007</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="G18" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="J18" s="5" t="s">
+      <c r="J18" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="K18" s="5" t="s">
+      <c r="K18" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5" t="s">
+      <c r="L18" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="O18" s="5"/>
-    </row>
-    <row r="19" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="5">
+      <c r="O18" s="8"/>
+    </row>
+    <row r="19" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="8">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="8">
         <v>2017</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="G19" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J19" s="5" t="s">
+      <c r="J19" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="K19" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5" t="s">
+      <c r="L19" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="O19" s="5"/>
-    </row>
-    <row r="20" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="5">
+      <c r="O19" s="8"/>
+    </row>
+    <row r="20" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="8">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="8">
         <v>2024</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="G20" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="J20" s="13" t="s">
+      <c r="J20" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="K20" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="L20" s="5" t="s">
+      <c r="L20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5" t="s">
+      <c r="M20" s="8"/>
+      <c r="N20" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="O20" s="5"/>
+      <c r="O20" s="8"/>
     </row>
     <row r="21" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="18"/>
     </row>
     <row r="22" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="7">
+      <c r="A22" s="2">
         <v>18</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="L22" s="7"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7" t="s">
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="O22" s="7"/>
-    </row>
-    <row r="23" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="7">
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="8">
         <v>19</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="J23" s="7" t="s">
+      <c r="J23" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7" t="s">
+      <c r="L23" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="O23" s="7"/>
-    </row>
-    <row r="24" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="7">
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="8">
         <v>20</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="E24" s="7">
+      <c r="E24" s="8">
         <v>2013</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="I24" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="J24" s="7" t="s">
+      <c r="J24" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K24" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7" t="s">
+      <c r="L24" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="O24" s="7"/>
-    </row>
-    <row r="25" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="7">
+      <c r="O24" s="8"/>
+    </row>
+    <row r="25" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="8">
         <v>21</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="8">
         <v>2017</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="I25" s="3" t="s">
+      <c r="I25" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="J25" s="7" t="s">
+      <c r="J25" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="K25" s="7" t="s">
+      <c r="K25" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L25" s="7"/>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7" t="s">
+      <c r="L25" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="O25" s="7"/>
-    </row>
-    <row r="26" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="7">
+      <c r="O25" s="8"/>
+    </row>
+    <row r="26" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="8">
         <v>22</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="8">
         <v>2001</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="I26" s="3" t="s">
+      <c r="I26" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="J26" s="7" t="s">
+      <c r="J26" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="K26" s="7" t="s">
+      <c r="K26" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7" t="s">
+      <c r="L26" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="O26" s="7"/>
-    </row>
-    <row r="27" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="7">
+      <c r="O26" s="8"/>
+    </row>
+    <row r="27" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="8">
         <v>23</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="8">
         <v>2022</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H27" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="J27" s="7" t="s">
+      <c r="J27" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="K27" s="7" t="s">
+      <c r="K27" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7" t="s">
+      <c r="L27" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="O27" s="7"/>
-    </row>
-    <row r="28" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="7">
+      <c r="O27" s="8"/>
+    </row>
+    <row r="28" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="8">
         <v>24</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="8">
         <v>2018</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I28" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="J28" s="7" t="s">
+      <c r="J28" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="K28" s="7" t="s">
+      <c r="K28" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7" t="s">
+      <c r="L28" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="O28" s="7"/>
-    </row>
-    <row r="29" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="7">
+      <c r="O28" s="8"/>
+    </row>
+    <row r="29" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="8">
         <v>25</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="8">
         <v>2012</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="J29" s="7" t="s">
+      <c r="J29" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="K29" s="7" t="s">
+      <c r="K29" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
-      <c r="N29" s="7" t="s">
+      <c r="L29" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="O29" s="7"/>
-    </row>
-    <row r="30" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="7">
+      <c r="O29" s="8"/>
+    </row>
+    <row r="30" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="8">
         <v>26</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="8">
         <v>2012</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I30" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="J30" s="7" t="s">
+      <c r="J30" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="K30" s="7" t="s">
+      <c r="K30" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="L30" s="7"/>
-      <c r="M30" s="7"/>
-      <c r="N30" s="7" t="s">
+      <c r="L30" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="O30" s="7"/>
+      <c r="O30" s="8"/>
     </row>
     <row r="31" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
-      <c r="N31" s="18"/>
-      <c r="O31" s="18"/>
-    </row>
-    <row r="32" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+    </row>
+    <row r="32" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="8">
         <v>27</v>
       </c>
@@ -2700,23 +3066,25 @@
       <c r="H32" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="I32" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="J32" s="8" t="s">
+      <c r="J32" s="13" t="s">
         <v>238</v>
       </c>
       <c r="K32" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L32" s="8"/>
+      <c r="L32" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="M32" s="8"/>
       <c r="N32" s="8" t="s">
         <v>239</v>
       </c>
       <c r="O32" s="8"/>
     </row>
-    <row r="33" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="8">
         <v>28</v>
       </c>
@@ -2726,7 +3094,7 @@
       <c r="C33" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="12" t="s">
         <v>241</v>
       </c>
       <c r="E33" s="8">
@@ -2741,7 +3109,7 @@
       <c r="H33" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I33" s="8" t="s">
         <v>245</v>
       </c>
       <c r="J33" s="8" t="s">
@@ -2750,14 +3118,16 @@
       <c r="K33" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="L33" s="8"/>
+      <c r="L33" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="M33" s="8"/>
       <c r="N33" s="8" t="s">
         <v>248</v>
       </c>
       <c r="O33" s="8"/>
     </row>
-    <row r="34" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:15" s="10" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="8">
         <v>29</v>
       </c>
@@ -2782,7 +3152,7 @@
       <c r="H34" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="8" t="s">
         <v>254</v>
       </c>
       <c r="J34" s="8" t="s">
@@ -2791,202 +3161,204 @@
       <c r="K34" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="L34" s="8"/>
+      <c r="L34" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="M34" s="8"/>
       <c r="N34" s="8" t="s">
         <v>257</v>
       </c>
       <c r="O34" s="8"/>
     </row>
-    <row r="35" spans="1:15" ht="57" x14ac:dyDescent="0.45">
-      <c r="A35" s="15">
+    <row r="35" spans="1:15" s="10" customFormat="1" ht="57" x14ac:dyDescent="0.45">
+      <c r="A35" s="14">
         <v>30</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="D35" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="E35" s="15">
+      <c r="E35" s="14">
         <v>2002</v>
       </c>
-      <c r="F35" s="15" t="s">
+      <c r="F35" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="G35" s="15" t="s">
+      <c r="G35" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="H35" s="15" t="s">
+      <c r="H35" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="I35" s="16" t="s">
+      <c r="I35" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="J35" s="19" t="s">
+      <c r="J35" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="K35" s="15" t="s">
+      <c r="K35" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="L35" s="15" t="s">
+      <c r="L35" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M35" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="M35" s="15" t="s">
+      <c r="N35" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="O35" s="14" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" s="10" customFormat="1" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A36" s="14">
+        <v>31</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="E36" s="14">
+        <v>2005</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="K36" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="L36" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M36" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="N35" s="15" t="s">
-        <v>266</v>
-      </c>
-      <c r="O35" s="15" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A36" s="15">
-        <v>31</v>
-      </c>
-      <c r="B36" s="15" t="s">
+      <c r="N36" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="O36" s="14" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" s="10" customFormat="1" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A37" s="14">
+        <v>32</v>
+      </c>
+      <c r="B37" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C36" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="E36" s="15">
-        <v>2005</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>260</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H36" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="I36" s="16" t="s">
+      <c r="C37" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E37" s="14">
+        <v>2018</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="G37" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="H37" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="I37" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="J36" s="15" t="s">
-        <v>271</v>
-      </c>
-      <c r="K36" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="L36" s="15" t="s">
+      <c r="J37" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="K37" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="L37" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M37" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="M36" s="15" t="s">
+      <c r="N37" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="O37" s="14" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" s="10" customFormat="1" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A38" s="14">
+        <v>33</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="E38" s="14">
+        <v>2019</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="K38" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="L38" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M38" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="N36" s="15" t="s">
-        <v>273</v>
-      </c>
-      <c r="O36" s="15" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A37" s="15">
-        <v>32</v>
-      </c>
-      <c r="B37" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>275</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="E37" s="15">
-        <v>2018</v>
-      </c>
-      <c r="F37" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="G37" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="H37" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="I37" s="16" t="s">
-        <v>262</v>
-      </c>
-      <c r="J37" s="15" t="s">
-        <v>278</v>
-      </c>
-      <c r="K37" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="L37" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="M37" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="N37" s="15" t="s">
-        <v>280</v>
-      </c>
-      <c r="O37" s="15" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A38" s="15">
-        <v>33</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>282</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>283</v>
-      </c>
-      <c r="E38" s="15">
-        <v>2019</v>
-      </c>
-      <c r="F38" s="15" t="s">
-        <v>284</v>
-      </c>
-      <c r="G38" s="15" t="s">
-        <v>285</v>
-      </c>
-      <c r="H38" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="I38" s="16" t="s">
-        <v>262</v>
-      </c>
-      <c r="J38" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="K38" s="15" t="s">
-        <v>288</v>
-      </c>
-      <c r="L38" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="M38" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="N38" s="15" t="s">
+      <c r="N38" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="O38" s="15" t="s">
+      <c r="O38" s="14" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:15" s="10" customFormat="1" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A39" s="15">
         <v>34</v>
       </c>
@@ -3011,7 +3383,7 @@
       <c r="H39" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="I39" s="16" t="s">
+      <c r="I39" s="15" t="s">
         <v>262</v>
       </c>
       <c r="J39" s="15" t="s">
@@ -3020,8 +3392,8 @@
       <c r="K39" s="15" t="s">
         <v>296</v>
       </c>
-      <c r="L39" s="15" t="s">
-        <v>265</v>
+      <c r="L39" s="12" t="s">
+        <v>25</v>
       </c>
       <c r="M39" s="15" t="s">
         <v>265</v>
@@ -3034,12 +3406,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A12:O12"/>
-    <mergeCell ref="A21:O21"/>
-    <mergeCell ref="A31:O31"/>
-    <mergeCell ref="A2:O2"/>
-  </mergeCells>
   <hyperlinks>
     <hyperlink ref="J3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="J20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -3048,8 +3414,18 @@
     <hyperlink ref="J4" r:id="rId5" xr:uid="{2909B6C9-E558-4A12-9BBE-0382A7154012}"/>
     <hyperlink ref="J5" r:id="rId6" xr:uid="{C465BD60-B7D2-4598-A019-13C4EB82C6F3}"/>
     <hyperlink ref="J11" r:id="rId7" xr:uid="{195D7C61-85E4-4BD4-83D3-3802693829D1}"/>
+    <hyperlink ref="J16" r:id="rId8" xr:uid="{9A16E595-22A5-4312-8334-2D78EEF8A33C}"/>
+    <hyperlink ref="J17" r:id="rId9" xr:uid="{8526C63B-668A-4656-AD56-1E1FE4F5020E}"/>
+    <hyperlink ref="J23" r:id="rId10" xr:uid="{54C9FDFC-B554-4F40-A9D2-7E12F1A8CBE1}"/>
+    <hyperlink ref="J24" r:id="rId11" xr:uid="{8AE6FB54-C074-4743-978F-F6AF3064D35A}"/>
+    <hyperlink ref="J25" r:id="rId12" xr:uid="{BFC747AB-F449-4761-B662-36E2CE7A53B3}"/>
+    <hyperlink ref="J32" r:id="rId13" xr:uid="{15B3863E-69C6-4407-99A9-7C4B78C1987F}"/>
+    <hyperlink ref="J19" r:id="rId14" xr:uid="{2016E98E-C46C-407F-8144-4ECAABD40570}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId15"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3063,15 +3439,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="3" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="4" t="s">
         <v>301</v>
       </c>
       <c r="B2" t="s">
@@ -3079,7 +3455,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="5" t="s">
         <v>303</v>
       </c>
       <c r="B3" t="s">
@@ -3087,7 +3463,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="6" t="s">
         <v>305</v>
       </c>
       <c r="B4" t="s">
@@ -3095,10 +3471,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="3" t="s">
         <v>308</v>
       </c>
     </row>
@@ -3135,34 +3511,34 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="3" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="3" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="3" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="3" t="s">
         <v>318</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Litteraturliste verifisert og korrigert: 14 PDFer, 13 metadatafiks
Nye PDFer (14): #35 Harchol-Balter, #37 APCO, #38 CalOES, #39 Penverne,
#40 Jamtli, #41 Riksrevisionen, #43 NTIA, #44 EU 112, #46 Aksin,
#47 Jouini, #48 Kim, #49 Byrsell (Swedish EMDC), #50 Samdal (Norway),
#51 Hart 2006

Korreksjoner verifisert mot PDF:
- #4 Koole: lagt til Mandelbaum som medforfatter
- #15 Restrepo: Henderson (ikke Ingolfsson)
- #17 Platou: ar markert som ikke verifisert
- #24: Justis- og politidepartementet (ikke DFO)
- #29: UK DSIT (ikke Ofcom), 2025
- #33 Vera: lagt til personforfattere
- #37 APCO: 2019 (ikke 2020)
- #39 Penverne: full korrekt tittel
- #40 Jamtli: full korrekt tittel
- #43 NTIA: full korrekt tittel
- #44 EU 112: full korrekt tittel
- #49 Swedish EMDC: Byrsell et al. (ikke Ellensen)
- #50 Norway dispatch: Samdal (ikke Rehn)
- #45 NENA-STA-045.1 fjernet (ikke relevant - om 988 mental helse)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
+++ b/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
@@ -54,8 +54,9 @@
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -99,8 +100,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
-        <bgColor rgb="00305496"/>
+        <fgColor rgb="FF305496"/>
+        <bgColor rgb="FF305496"/>
       </patternFill>
     </fill>
   </fills>
@@ -173,7 +174,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -208,7 +209,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -943,27 +946,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="11.53125" customWidth="1" min="12" max="12"/>
-    <col width="16.19921875" customWidth="1" min="13" max="13"/>
-    <col width="55" customWidth="1" min="14" max="14"/>
-    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" style="18" min="1" max="1"/>
+    <col width="18" customWidth="1" style="18" min="2" max="2"/>
+    <col width="30" customWidth="1" style="18" min="3" max="3"/>
+    <col width="45" customWidth="1" style="18" min="4" max="4"/>
+    <col width="6" customWidth="1" style="18" min="5" max="5"/>
+    <col width="28" customWidth="1" style="18" min="6" max="6"/>
+    <col width="18" customWidth="1" style="18" min="7" max="7"/>
+    <col width="45" customWidth="1" style="18" min="8" max="8"/>
+    <col width="29.265625" customWidth="1" style="18" min="9" max="9"/>
+    <col width="35" customWidth="1" style="18" min="10" max="10"/>
+    <col width="16" customWidth="1" style="18" min="11" max="11"/>
+    <col width="11.53125" customWidth="1" style="18" min="12" max="12"/>
+    <col width="16.19921875" customWidth="1" style="18" min="13" max="13"/>
+    <col width="55" customWidth="1" style="18" min="14" max="14"/>
+    <col width="35" customWidth="1" style="18" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="30" customHeight="1" s="18">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Nr</t>
@@ -1040,7 +1043,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="18" customHeight="1" s="18">
       <c r="A2" s="7" t="inlineStr">
         <is>
           <t>KATEGORI 1: Metodisk kjernelitteratur – Erlang-C / Køteori</t>
@@ -1253,7 +1256,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Koole, G.</t>
+          <t>Koole, G., &amp; Mandelbaum, A.</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -1302,10 +1305,14 @@
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>Koole, G. (2002). Queueing models of call centers: An introduction. [Sjekk versjon og publiseringsdetaljer]</t>
-        </is>
-      </c>
-      <c r="O6" s="8" t="n"/>
+          <t>Koole, G., &amp; Mandelbaum, A. (2002). Queueing models of call centers: An introduction. Annals of Operations Research, 113(1-4), 41-59. https://doi.org/10.1023/A:1020949626017</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: Lagt til Mandelbaum som andre forfatter (manglet i original).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customFormat="1" customHeight="1" s="10">
       <c r="A7" s="8" t="n">
@@ -1632,7 +1639,7 @@
       </c>
       <c r="O11" s="8" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="18" customHeight="1" s="18">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>KATEGORI 2: Nødmeldesentral-spesifikk litteratur (110 / 112 / EMS)</t>
@@ -1975,7 +1982,7 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Restrepo, M., Ingolfsson, A., &amp; Topaloglu, H.</t>
+          <t>Restrepo, M., Henderson, S. G., &amp; Topaloglu, H.</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -2024,10 +2031,14 @@
       <c r="M18" s="8" t="n"/>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>Restrepo, M., Ingolfsson, A., &amp; Topaloglu, H. (2007). [Tittel og detaljer må verifiseres]</t>
-        </is>
-      </c>
-      <c r="O18" s="8" t="n"/>
+          <t>Restrepo, M., Henderson, S. G., &amp; Topaloglu, H. (2009). Erlang loss models for the static deployment of ambulances. Health Care Management Science, 12(1), 67-79. https://doi.org/10.1007/s10729-008-9077-4</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: Forfatter endret fra Ingolfsson til Henderson (var feil i originalen). Verifisert mot PDF.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customFormat="1" customHeight="1" s="10">
       <c r="A19" s="8" t="n">
@@ -2133,7 +2144,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>❌ Ikke verifisert – søk i NVA / Cristin</t>
+          <t>Year ikke verifisert mot forside - sannsynligvis 2023 eller tidlig 2024 basert pa studieperiode 2021-2023</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
@@ -2157,16 +2168,20 @@
           <t>Platou, H. C. S. (2024). Videosamtale på AMK [Masteroppgave]. Ikke verifisert.</t>
         </is>
       </c>
-      <c r="O20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: Aret ble ikke funnet pa forsiden. Trenger verifikasjon mot UiO DUO arkiv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="18">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>KATEGORI 3: Norsk/nordisk offentlig og grå litteratur</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="60" customHeight="1" s="18">
       <c r="A22" s="2" t="n">
         <v>18</v>
       </c>
@@ -2567,7 +2582,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Direktoratet for forvaltning og økonomistyring (DFØ)</t>
+          <t>Justis- og politidepartementet (interdepartemental arbeidsgruppe)</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -2616,10 +2631,14 @@
       <c r="M28" s="8" t="n"/>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>Direktoratet for forvaltning og økonomistyring. (2018). [Tittel og detaljer – verifiser].</t>
-        </is>
-      </c>
-      <c r="O28" s="8" t="n"/>
+          <t>Justis- og politidepartementet. (2009). Forslag til fremtidig organisering av nodmeldetjenesten: Rapport fra en interdepartemental arbeidsgruppe. Justis- og politidepartementet.</t>
+        </is>
+      </c>
+      <c r="O28" s="8" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: Forfatter endret fra DFO til Justis- og politidepartementet (interdepartemental arbeidsgruppe). DFO er ikke involvert.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="60" customFormat="1" customHeight="1" s="10">
       <c r="A29" s="8" t="n">
@@ -2751,7 +2770,7 @@
       </c>
       <c r="O30" s="8" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
+    <row r="31" ht="18" customHeight="1" s="18">
       <c r="A31" s="7" t="inlineStr">
         <is>
           <t>KATEGORI 4: Internasjonale standarder og servicegrad</t>
@@ -2899,12 +2918,12 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Ofcom</t>
+          <t>Department for Science, Innovation &amp; Technology (UK)</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>PECS Code of Practice – Version 1.1</t>
+          <t>Public Emergency Call Service - Code of Practice (Version 1.1)</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
@@ -2912,7 +2931,7 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>Ofcom regulatorisk dokument (UK)</t>
+          <t>Department for Science, Innovation &amp; Technology, June 2025</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -2948,10 +2967,14 @@
       <c r="M34" s="8" t="n"/>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>Ofcom. (2025). PECS code of practice – version 1.1. Ofcom. [Verifiser tilgjengelighet].</t>
-        </is>
-      </c>
-      <c r="O34" s="8" t="n"/>
+          <t>Department for Science, Innovation &amp; Technology. (2025). Public emergency call service: Code of practice (Version 1.1). UK Government.</t>
+        </is>
+      </c>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: Forfatter endret fra Ofcom til Department for Science, Innovation &amp; Technology (UK). Ar 2025 (juni).</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="57" customFormat="1" customHeight="1" s="10">
       <c r="A35" s="14" t="n">
@@ -3183,7 +3206,7 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>Vera Institute of Justice</t>
+          <t>Neusteter, S. R., Mapolski, M., Khogali, M., &amp; O'Toole, M.</t>
         </is>
       </c>
       <c r="D38" s="14" t="inlineStr">
@@ -3236,12 +3259,12 @@
       </c>
       <c r="N38" s="14" t="inlineStr">
         <is>
-          <t>Vera Institute of Justice. (2019). The 911 call processing system: A review of the literature as it relates to policing. Vera Institute of Justice.</t>
+          <t>Neusteter, S. R., Mapolski, M., Khogali, M., &amp; O'Toole, M. (2019). The 911 call processing system: A review of the literature as it relates to policing. Vera Institute of Justice.</t>
         </is>
       </c>
       <c r="O38" s="14" t="inlineStr">
         <is>
-          <t>Nyttig i diskusjon og begrensninger: Erlang-C modellerer bare anropsmottak, ikke hele operasjonsforløpet.</t>
+          <t>KORRIGERT 2026-04-08: Lagt til personforfattere (var bare korporativ Vera Institute tidligere). Juli 2019.</t>
         </is>
       </c>
     </row>
@@ -3318,81 +3341,81 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="16" t="inlineStr">
+    <row r="40" ht="15.75" customHeight="1" s="18">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>KATEGORI 5: Tilleggssok april 2026 - team-basert kapasitet, degradert drift og bemanningskrise</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="n">
+    <row r="41" customFormat="1" s="10">
+      <c r="A41" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>Koteori - multiserver jobs</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Harchol-Balter, M.</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="10" t="inlineStr">
         <is>
           <t>The multiserver job queueing model</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="10" t="inlineStr">
         <is>
           <t>Queueing Systems, 100, 201-203</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert teoriartikkel</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="10" t="inlineStr">
         <is>
           <t>KRITISK for kap 3 og kap 6: gir det matematiske spraket for makkerpar - jobber som krever n_i samtidige servere parallelt. Stabilitetsregion er mindre enn idealiserte M/M/c-grenser pga. fragmentering.</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert - verifiser DOI og forfatterattribusjon</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s11134-022-09762-x</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="10" t="inlineStr">
         <is>
           <t>Sjekk Springer (institusjonell tilgang HiMolde)</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
+      <c r="L41" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M41" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 3 og 6</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="N41" s="10" t="inlineStr">
         <is>
           <t>Harchol-Balter, M. (2022). The multiserver job queueing model. Queueing Systems, 100, 201-203. https://doi.org/10.1007/s11134-022-09762-x</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O41" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Direkte teoretisk forankring for makkerpar-konseptet.</t>
         </is>
@@ -3440,7 +3463,7 @@
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="16" t="inlineStr">
         <is>
           <t>https://doi.org/10.1287/mnsc.30.1.51</t>
         </is>
@@ -3452,7 +3475,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>NEI</t>
+          <t>BESTILLES via HiMolde - bak betalingsmur</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3471,366 +3494,366 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="n">
+    <row r="43" customFormat="1" s="10">
+      <c r="A43" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>PSAP empiri / staffing</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>APCO International / CSSR</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
         <is>
           <t>Call Handling and Incident Processing in Emergency Communications Centers</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v>2020</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>APCO Project Report (Survey N=772 PSAP-ansatte)</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="E43" s="10" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>APCO International / George Mason University Center for Social Science Research, September 2019</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
         <is>
           <t>Bransjerapport / survey</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="10" t="inlineStr">
         <is>
           <t>Empirisk stotte for at bemanning (rapportert av 65,4 % av sentre) og duplikatanrop forsinker prosesseringstid. Direkte stotte for V1, V2 og V3.</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="13" t="inlineStr">
         <is>
           <t>https://www.apcointl.org/~documents/report/incident-handling-eccs-2020</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="10" t="inlineStr">
         <is>
           <t>Apen PDF (APCO)</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
+      <c r="L43" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M43" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 8 diskusjon</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>APCO International. (2020). Call handling and incident processing in emergency communications centers. APCO International / Center for Statistics and Sustainability Research.</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
+      <c r="N43" s="10" t="inlineStr">
+        <is>
+          <t>APCO International. (2019). Call handling and incident processing in emergency communications centers: A research report. APCO International / George Mason University Center for Social Science Research.</t>
+        </is>
+      </c>
+      <c r="O43" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Stor survey (N=772). Beste empiriske stotte for bemanning som forsinkelsesfaktor.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="n">
+    <row r="44" customFormat="1" s="10">
+      <c r="A44" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>Bemanningskrise / staffing</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>California Governor's Office of Emergency Services (CalOES)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>California PSAP and Staffing Study 2024</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>Offentlig statsrapport, California</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="10" t="inlineStr">
         <is>
           <t>Offentlig rapport</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="10" t="inlineStr">
         <is>
           <t>Konkret tall: 19 % gjennomsnittlig vacancy rate blant californiske PSAP-er. Brukes som referanse for 'bemanningskrise'-argumentet i diskusjonen.</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="13" t="inlineStr">
         <is>
           <t>https://www.caloes.ca.gov/wp-content/uploads/PSC/Documents/CalOES-2024-Staffing-Study.pdf</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="10" t="inlineStr">
         <is>
           <t>Apen PDF (CalOES)</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
+      <c r="L44" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M44" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 8 (kontekst)</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="N44" s="10" t="inlineStr">
         <is>
           <t>California Governor's Office of Emergency Services. (2024). California PSAP and staffing study 2024. CalOES.</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="O44" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Internasjonal kontekst for bemanningsproblemer.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="n">
+    <row r="45" customFormat="1" s="10">
+      <c r="A45" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Pooling / digital twin</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Penverne, Y., m.fl.</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>A digital twin for emergency medical communication centers</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Penverne, Y., Martinez, C., Cellier, N., Pehlivan, C., Jenvrin, J., Savary, D., Debierre, V., Deciron, F., Bichri, A., Lebastard, Q., Montassier, E., Leclere, B., &amp; Fontanili, F.</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>A simulation based digital twin approach to assessing the organization of response to emergency calls</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>npj Digital Medicine</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>npj Digital Medicine, 7, 385</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert simuleringsstudie</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="10" t="inlineStr">
         <is>
           <t>Tester dekompartmentalisering/pooling mellom EMCC-sentre, viser 17-21 % forbedring i servicekvalitet. Relevant for diskusjon av alternative dimensjoneringsstrategier.</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41746-024-01392-2</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="10" t="inlineStr">
         <is>
           <t>Open access (Nature/npj)</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
+      <c r="L45" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M45" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 8 (alternativer)</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Penverne, Y., m.fl. (2024). A digital twin for emergency medical communication centers. npj Digital Medicine.</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
+      <c r="N45" s="10" t="inlineStr">
+        <is>
+          <t>Penverne, Y., Martinez, C., Cellier, N., Pehlivan, C., Jenvrin, J., Savary, D., Debierre, V., Deciron, F., Bichri, A., Lebastard, Q., Montassier, E., Leclere, B., &amp; Fontanili, F. (2024). A simulation based digital twin approach to assessing the organization of response to emergency calls. npj Digital Medicine, 7, 385. https://doi.org/10.1038/s41746-024-01392-2</t>
+        </is>
+      </c>
+      <c r="O45" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Verifiser fullt forfatternavn.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
+    <row r="46" customFormat="1" s="10">
+      <c r="A46" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Norsk nodmeldetjeneste</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Jamtli, B., m.fl.</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Decision-making in stroke calls at the Oslo emergency medical communication center</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Jamtli, B., Svendsen, E. J., Jorgensen, T. M., Kramer-Johansen, J., Hov, M. R., &amp; Hardeland, C.</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Factors affecting emergency medical dispatchers decision making in stroke calls — a qualitative study</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>BMC Emergency Medicine</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>BMC Emergency Medicine, 24, 214</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert kvalitativ studie</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="10" t="inlineStr">
         <is>
           <t>Norsk 113/AMK-kontekst. Beslutningstaking under tidspress, regulatoriske svartidskrav (90 % innen 10 sek), bruk av Norwegian Index. Brukes som norsk parallell.</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/s12873-024-01129-0</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="10" t="inlineStr">
         <is>
           <t>Open access (BMC)</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
+      <c r="L46" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M46" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 2 og 8</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>Jamtli, B., m.fl. (2024). Decision-making in stroke calls at the Oslo emergency medical communication center. BMC Emergency Medicine.</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
+      <c r="N46" s="10" t="inlineStr">
+        <is>
+          <t>Jamtli, B., Svendsen, E. J., Jorgensen, T. M., Kramer-Johansen, J., Hov, M. R., &amp; Hardeland, C. (2024). Factors affecting emergency medical dispatchers decision making in stroke calls — a qualitative study. BMC Emergency Medicine, 24, 214. https://doi.org/10.1186/s12873-024-01129-0</t>
+        </is>
+      </c>
+      <c r="O46" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Verifiser fullt forfatternavn og DOI.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="n">
+    <row r="47" customFormat="1" s="10">
+      <c r="A47" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>Governance / svartider</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
         <is>
           <t>Riksrevisionen (Sverige)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="10" t="inlineStr">
         <is>
           <t>Statens ansvar for 112 - Rapport RiR 2023:22 (sammanfattning)</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="10" t="inlineStr">
         <is>
           <t>Riksrevisionen, Sverige</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="10" t="inlineStr">
         <is>
           <t>Revisjonsrapport</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="10" t="inlineStr">
         <is>
           <t>KRITISK for kap 8: SOS Alarm har ikke nadd svartidsmal pa 10 ar. Sterkt belegg for at 'degradert drift' kan bli vedvarende tilstand, ikke unntak.</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="13" t="inlineStr">
         <is>
           <t>https://www.riksrevisionen.se/download/18.3ad2ec4c19329a0a7e56315/1731922695598/RiR_2023_22_summary.pdf</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="10" t="inlineStr">
         <is>
           <t>Apen PDF (Riksrevisionen)</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
+      <c r="L47" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M47" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 8 governance</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="N47" s="10" t="inlineStr">
         <is>
           <t>Riksrevisionen. (2023). Statens ansvar for 112 (RiR 2023:22). Riksrevisionen.</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O47" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Nordisk parallell. Sterk for governance-perspektiv.</t>
         </is>
@@ -3847,651 +3870,656 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NASA Ames Research Center</t>
+          <t>Hart, S. G., &amp; Staveland, L. E.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>NASA Task Load Index (NASA-TLX)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>oppdatert</t>
-        </is>
+          <t>Development of NASA-TLX (Task Load Index): Results of empirical and theoretical research</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1988</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>NASA Human Performance Research Group</t>
+          <t>I P. A. Hancock &amp; N. Meshkati (Red.), Advances in Psychology, 52, 139-183. North-Holland</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Metodebeskrivelse</t>
+          <t>Bokkapittel (kanonisk metodereferanse)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Etablert workload-maling. Gir metodisk forankring for 'solo-drift gir hoyere kognitiv belastning'-argumentet i kap 6.4 og 8.</t>
+          <t>Originalartikkelen som introduserte NASA-TLX som standardisert workload-malingsverktoy. Kanonisk referanse i all litteratur om kognitiv belastning. Brukes for a forankre 'solo-drift gir hoyere workload'-argumentet i kap 6.4 og 8.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
+          <t>Verifiser via Google Scholar</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0166-4115(08)62386-9</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Open access via flere arkiver (Google Scholar)</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>BESTILLES via HiMolde - bak betalingsmur</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Planlagt - kap 3, 8</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Hart, S. G., &amp; Staveland, L. E. (1988). Development of NASA-TLX (Task Load Index): Results of empirical and theoretical research. I P. A. Hancock &amp; N. Meshkati (Red.), Advances in Psychology (Vol. 52, s. 139-183). North-Holland.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Tilleggssok 2026-04-07. Kanonisk metodereferanse - erstatter NASA Ames sidereferanse. Sok 'Hart Staveland 1988 NASA-TLX' i Google Scholar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" customFormat="1" s="10">
+      <c r="A49" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>AI / future tech</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>National Telecommunications and Information Administration (NTIA)</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Improving 9-1-1 Operations with Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>NTIA, US Department of Commerce</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>Offentlig program/policy</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>Behandles som mulig framtidig scenario, ikke etablert effekt. Relevant for kort omtale i kap 8 om 'andre losninger pa kapasitetspress'.</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>https://humansystems.arc.nasa.gov/groups/TLX/</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Apen NASA-side</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>Planlagt - kap 3, 8</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>NASA Ames Research Center. (u.a.). NASA Task Load Index (NASA-TLX). Human Performance Research Group.</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>Tilleggssok 2026-04-07. Standard metode for kognitiv workload.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>43</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>AI / future tech</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>National Telecommunications and Information Administration (NTIA)</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>AI-Powered Call Triage for Next Generation 911</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ntia.gov/category/next-generation-911/improving-911-operations-with-artificial-intelligence</t>
+        </is>
+      </c>
+      <c r="K49" s="10" t="inlineStr">
+        <is>
+          <t>Apen NTIA-side</t>
+        </is>
+      </c>
+      <c r="L49" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M49" s="10" t="inlineStr">
+        <is>
+          <t>Vurderes - kap 8 (perspektiv)</t>
+        </is>
+      </c>
+      <c r="N49" s="10" t="inlineStr">
+        <is>
+          <t>National Telecommunications and Information Administration. (2024). Improving 9-1-1 operations with artificial intelligence. NTIA, Office of Public Safety Communications, U.S. Department of Commerce.</t>
+        </is>
+      </c>
+      <c r="O49" s="10" t="inlineStr">
+        <is>
+          <t>Tilleggssok 2026-04-07. Lavere prioritet - kun for perspektiv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" customFormat="1" s="10">
+      <c r="A50" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>EU statistikk / volum</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>European Commission</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Report from the Commission to the European Parliament and the Council on the effectiveness of the implementation of the single European emergency number '112' (COM(2024) 575 final)</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>NTIA, US Department of Commerce</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Offentlig program/policy</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Behandles som mulig framtidig scenario, ikke etablert effekt. Relevant for kort omtale i kap 8 om 'andre losninger pa kapasitetspress'.</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>European Commission</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
+        <is>
+          <t>Offentlig rapport</t>
+        </is>
+      </c>
+      <c r="H50" s="10" t="inlineStr">
+        <is>
+          <t>112-anrop okte til 176 millioner i 2023 (15 % okning vs 2021). Underbygger at volum- og tilgjengelighetsutfordringer er systemiske.</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
         <is>
           <t>Ikke verifisert</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>https://www.ntia.gov/category/next-generation-911/improving-911-operations-with-artificial-intelligence</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Apen NTIA-side</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Vurderes - kap 8 (perspektiv)</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>National Telecommunications and Information Administration. (2024). AI-powered call triage for Next Generation 911. NTIA, U.S. Department of Commerce.</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>Tilleggssok 2026-04-07. Lavere prioritet - kun for perspektiv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>44</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>EU statistikk / volum</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>European Commission</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Report on the implementation of the universal service obligation for emergency communications (COM(2024) 575)</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>European Commission</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Offentlig rapport</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>112-anrop okte til 176 millioner i 2023 (15 % okning vs 2021). Underbygger at volum- og tilgjengelighetsutfordringer er systemiske.</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>Ikke verifisert</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
+      <c r="J50" s="13" t="inlineStr">
         <is>
           <t>https://eur-lex.europa.eu/legal-content/EN/TXT/HTML/?uri=CELEX:52024DC0575</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="10" t="inlineStr">
         <is>
           <t>Apen EUR-Lex</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
+      <c r="L50" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M50" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 1 eller 8 (volumkontekst)</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>European Commission. (2024). Report on the implementation of the universal service obligation for emergency communications (COM(2024) 575). European Commission.</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
+      <c r="N50" s="10" t="inlineStr">
+        <is>
+          <t>European Commission. (2024). Report from the Commission to the European Parliament and the Council on the effectiveness of the implementation of the single European emergency number '112' (COM(2024) 575 final). European Commission.</t>
+        </is>
+      </c>
+      <c r="O50" s="10" t="inlineStr">
         <is>
           <t>Tilleggssok 2026-04-07. Brukes som internasjonal volumkontekst.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>45</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Tidsstandard / NENA</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>National Emergency Number Association (NENA)</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>NENA Standard for the Implementation of NG9-1-1 (NENA-STA-045.1-202X)</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>2025</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>NENA</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Nyere NENA-standard for NG9-1-1. Supplerer NENA-STA-020.1-2020. Vurderes for kap 3.6 (norsk kontekst og standarder).</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Ikke verifisert - sjekk endelig nummer</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>https://cdn.ymaws.com/www.nena.org/resource/resmgr/standards/NENA-STA-045.1-202Y_911-988_.pdf</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Apen NENA</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>Vurderes - kap 3</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>National Emergency Number Association. (2025). NENA standard for the implementation of NG9-1-1 (NENA-STA-045.1-202X). NENA.</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>Tilleggssok 2026-04-07. Lavere prioritet enn NENA-STA-020.1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
+    <row r="51" customFormat="1" s="10">
+      <c r="A51" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Kanonisk koteori (manglende)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>Aksin, Z., Armony, M., &amp; Mehrotra, V.</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D51" s="10" t="inlineStr">
         <is>
           <t>The modern call center: A multi-disciplinary perspective on operations management research</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E51" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F51" s="10" t="inlineStr">
         <is>
           <t>Production and Operations Management, 16(6), 665-688</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert review</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H51" s="10" t="inlineStr">
         <is>
           <t>Kanonisk modern call center review. Bor vaere med i kap 2 og 3 som referanse for hvordan feltet har utviklet seg etter Gans/Koole/Mandelbaum 2003.</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I51" s="10" t="inlineStr">
         <is>
           <t>Verifisert i komplett v1</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J51" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/j.1937-5956.2007.tb00288.x</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K51" s="10" t="inlineStr">
         <is>
           <t>Wiley (institusjonell tilgang)</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
+      <c r="L51" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M51" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 2, 3</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="N51" s="10" t="inlineStr">
         <is>
           <t>Aksin, Z., Armony, M., &amp; Mehrotra, V. (2007). The modern call center: A multi-disciplinary perspective on operations management research. Production and Operations Management, 16(6), 665-688.</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="O51" s="10" t="inlineStr">
         <is>
           <t>Manglet i nedlastinger. Identifisert i komplett v1 (2026-03-29).</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="n">
+    <row r="52" customFormat="1" s="10">
+      <c r="A52" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Team-basert ko (manglende)</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
         <is>
           <t>Jouini, O., Dallery, Y., &amp; Nait-Abdallah, R.</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>Analysis of the impact of team-based organizations in call center management</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E52" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F52" s="10" t="inlineStr">
         <is>
           <t>Management Science, 54(2), 400-414</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G52" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert artikkel</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H52" s="10" t="inlineStr">
         <is>
           <t>KRITISK for makkerpar-argumentet. Den eneste tidligere studien som direkte modellerer team-basert organisering i call center. Bor vaere sentral i kap 3.5.</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I52" s="10" t="inlineStr">
         <is>
           <t>Verifisert i komplett v1 (DOI rettet)</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J52" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1287/mnsc.1070.0822</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K52" s="10" t="inlineStr">
         <is>
           <t>INFORMS (institusjonell tilgang)</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
+      <c r="L52" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M52" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 3.5</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="N52" s="10" t="inlineStr">
         <is>
           <t>Jouini, O., Dallery, Y., &amp; Nait-Abdallah, R. (2008). Analysis of the impact of team-based organizations in call center management. Management Science, 54(2), 400-414.</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="O52" s="10" t="inlineStr">
         <is>
           <t>Manglet i nedlastinger. Komplett v1 rettet DOI fra .0792 til .0822.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="n">
+    <row r="53" customFormat="1" s="10">
+      <c r="A53" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>Cooperating servers (manglende)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>Kim, C., Lee, M., Dudin, A., &amp; Klimenok, V.</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>Multi-server queueing systems with cooperation of the servers</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E53" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F53" s="10" t="inlineStr">
         <is>
           <t>Annals of Operations Research, 162(1), 57-68</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert artikkel</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H53" s="10" t="inlineStr">
         <is>
           <t>KRITISK: ko-modeller med 'cooperation of servers' er den naermeste matematiske analogien til makkerpar for Harchol-Balter 2022.</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I53" s="10" t="inlineStr">
         <is>
           <t>Verifisert i komplett v1</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="J53" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s10479-008-0319-0</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K53" s="10" t="inlineStr">
         <is>
           <t>Springer (institusjonell tilgang)</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
+      <c r="L53" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M53" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 3.5</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="N53" s="10" t="inlineStr">
         <is>
           <t>Kim, C., Lee, M., Dudin, A., &amp; Klimenok, V. (2008). Multi-server queueing systems with cooperation of the servers. Annals of Operations Research, 162(1), 57-68.</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="O53" s="10" t="inlineStr">
         <is>
           <t>Manglet i nedlastinger. Identifisert i komplett v1 (2026-03-29).</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="n">
+    <row r="54" customFormat="1" s="10">
+      <c r="A54" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>Nordisk EMDC (manglende - verifiser)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Ellensen, E. N., Sunde, K., Haugland, G., m.fl.</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Swedish emergency medical dispatch centres' ability to answer emergency medical calls</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>Byrsell, F., Jonsson, M., Claesson, A., Ringh, M., Svensson, L., Riva, G., Nordberg, P., Forsberg, S., Hollenberg, J., &amp; Nord, A.</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Swedish emergency medical dispatch centres' ability to answer emergency medical calls and dispatch an ambulance in response to out-of-hospital cardiac arrest calls in accordance with the American Heart Association performance goals: An observational study</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F54" s="10" t="inlineStr">
         <is>
           <t>Resuscitation, 189, artikkel 109896</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G54" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert observasjonsstudie</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H54" s="10" t="inlineStr">
         <is>
           <t>Nordisk EMDC-svartidsstudie. Direkte sammenlignbar med var norske kontekst.</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>NB: ChatGPT-tilleggssok siterer dette som 'Byrsell et al. 2023' med samme DOI. VERIFISER hvem som er forfatter.</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>Verifisert mot PDF 2026-04-08 - forfattere er Byrsell et al., ikke Ellensen</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.resuscitation.2023.109896</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="K54" s="10" t="inlineStr">
         <is>
           <t>Elsevier (institusjonell tilgang)</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
+      <c r="L54" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M54" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 2, 3, 8</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>[Verifiser forfatter] (2023). Swedish emergency medical dispatch centres' ability to answer emergency medical calls. Resuscitation, 189, artikkel 109896.</t>
-        </is>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>Konflikt mellom v1 (Ellensen) og tilleggssok (Byrsell). Sjekk PubMed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
+      <c r="N54" s="10" t="inlineStr">
+        <is>
+          <t>Byrsell, F., Jonsson, M., Claesson, A., Ringh, M., Svensson, L., Riva, G., Nordberg, P., Forsberg, S., Hollenberg, J., &amp; Nord, A. (2023). Swedish emergency medical dispatch centres' ability to answer emergency medical calls and dispatch an ambulance in response to out-of-hospital cardiac arrest calls in accordance with the American Heart Association performance goals: An observational study. Resuscitation, 189, 109896. https://doi.org/10.1016/j.resuscitation.2023.109896</t>
+        </is>
+      </c>
+      <c r="O54" s="10" t="inlineStr">
+        <is>
+          <t>Tilleggssok 2026-04-07. KORRIGERT 2026-04-08: forfatterne er Byrsell et al., ikke Ellensen som tidligere oppfort. Verifisert mot PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" customFormat="1" s="10">
+      <c r="A55" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Norsk EMS (manglende)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Rehn, M., Samdal, M., Magnusson, V., m.fl.</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Dispatch accuracy of physician-staffed emergency medical services in trauma care in South-East Norway</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>Samdal, M., Thorsen, K., Graesli, O., Sandberg, M., &amp; Rehn, M.</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Dispatch accuracy of physician-staffed emergency medical services in trauma care in south-east Norway: A retrospective observational study</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F55" s="10" t="inlineStr">
         <is>
           <t>Scandinavian Journal of Trauma, Resuscitation and Emergency Medicine, 29, artikkel 169</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G55" s="10" t="inlineStr">
         <is>
           <t>Fagfellevurdert studie</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H55" s="10" t="inlineStr">
         <is>
           <t>Norsk dispatch-noyaktighet. Relevant for kap 2 og 8 som norsk referanse.</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Verifisert i komplett v1</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>Verifisert mot PDF 2026-04-08 - hovedforfatter er Samdal, ikke Rehn</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/s13049-021-00982-3</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K55" s="10" t="inlineStr">
         <is>
           <t>Open access (BMC)</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>NEI</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
+      <c r="L55" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M55" s="10" t="inlineStr">
         <is>
           <t>Planlagt - kap 2</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>Rehn, M., Samdal, M., Magnusson, V., Lindner, T., Lossius, H. M., &amp; Soreide, E. (2021). Dispatch accuracy of physician-staffed emergency medical services in trauma care in South-East Norway. Scandinavian Journal of Trauma, Resuscitation and Emergency Medicine, 29, 169.</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>Manglet i nedlastinger. Komplett v1 rettet art.nr fra 163 til 169.</t>
+      <c r="N55" s="10" t="inlineStr">
+        <is>
+          <t>Samdal, M., Thorsen, K., Graesli, O., Sandberg, M., &amp; Rehn, M. (2021). Dispatch accuracy of physician-staffed emergency medical services in trauma care in south-east Norway: A retrospective observational study. Scandinavian Journal of Trauma, Resuscitation and Emergency Medicine, 29, 169. https://doi.org/10.1186/s13049-021-00982-3</t>
+        </is>
+      </c>
+      <c r="O55" s="10" t="inlineStr">
+        <is>
+          <t>KORRIGERT 2026-04-08: hovedforfatter er Samdal, ikke Rehn. Verifisert mot PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" customFormat="1" s="10">
+      <c r="A56" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Workload / metodikk</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>Hart, S. G.</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>NASA-Task Load Index (NASA-TLX); 20 years later</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="n">
+        <v>2006</v>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>Proceedings of the Human Factors and Ergonomics Society Annual Meeting, 50(9), 904-908</t>
+        </is>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>Konferansepublikasjon (oppfolger til 1988)</t>
+        </is>
+      </c>
+      <c r="H56" s="10" t="inlineStr">
+        <is>
+          <t>Hart's egen retrospektive evaluering av NASA-TLX 20 ar etter introduksjonen. Bekrefter verktoyets validitet og dokumenterer hvordan det brukes i ulike domener. Brukes som supplement til 1988-referansen.</t>
+        </is>
+      </c>
+      <c r="I56" s="10" t="inlineStr">
+        <is>
+          <t>Verifiser DOI</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/154193120605000909</t>
+        </is>
+      </c>
+      <c r="K56" s="10" t="inlineStr">
+        <is>
+          <t>SAGE (institusjonell tilgang HiMolde)</t>
+        </is>
+      </c>
+      <c r="L56" s="10" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M56" s="10" t="inlineStr">
+        <is>
+          <t>Vurderes - kap 3, 8</t>
+        </is>
+      </c>
+      <c r="N56" s="10" t="inlineStr">
+        <is>
+          <t>Hart, S. G. (2006). NASA-Task Load Index (NASA-TLX); 20 years later. Proceedings of the Human Factors and Ergonomics Society Annual Meeting, 50(9), 904-908. https://doi.org/10.1177/154193120605000909</t>
+        </is>
+      </c>
+      <c r="O56" s="10" t="inlineStr">
+        <is>
+          <t>Tilleggssok 2026-04-07. Brukes sammen med Hart &amp; Staveland 1988 om mer dokumentasjon trengs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" customFormat="1" s="10">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/154193120605000909</t>
         </is>
       </c>
     </row>
@@ -4514,10 +4542,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4531,8 +4575,8 @@
   <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" style="18" min="1" max="1"/>
+    <col width="60" customWidth="1" style="18" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
V3-kategorier konsistent i kap 5-7: erstatter A/B/C/D med D/S/L-aba/L-hendelse/L-ukjent/F/V
- kap 5: tabell 5.1 inkluderer variant A+B, analyseenhet oppdatert, variabeltabell med riktige BRIS-felt
- kap 6.2: omskrevet fra abstrakt A/B/C/D til operativ V3-klassifisering med BRIS-regler
- kap 6.5: fjernet duplisert klassifiseringstabell (nå i 6.2), seksjonsnumre justert
- kap 7: alle A/B/C-referanser erstattet med V3-kategorinavn og pekere til variant B

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
+++ b/012 fase 2 - plan/Litteraturliste_LOG650_G20_Rune.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be25ac4905db4876/Documents/Skole utdanning/Logistikk studie/LOG650 LOGISTIKK OG KI/G20-rune-individuell/012 fase 2 - plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_55A7D5BCD010BC39C101FC9027789992ED30C35C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38CC5CED-A79C-4188-9EC9-6D9400FDF237}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_55A7D5BCD010BC39C101FC9027789992ED30C35C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30A4575F-D04F-4504-8238-EE1FA822012F}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="62385" yWindow="7095" windowWidth="16200" windowHeight="9315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Litteraturliste" sheetId="1" r:id="rId1"/>
@@ -2723,8 +2723,8 @@
     <col min="10" max="10" width="35" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="11.53125" customWidth="1"/>
-    <col min="13" max="13" width="16.19921875" customWidth="1"/>
-    <col min="14" max="14" width="55" customWidth="1"/>
+    <col min="13" max="13" width="36.19921875" customWidth="1"/>
+    <col min="14" max="14" width="101.53125" customWidth="1"/>
     <col min="15" max="15" width="35" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>